<commit_message>
GRTS a partir de poligons
Prova per aplicar GRTS a partir de poligons, de moment no ens convennç i seguirem fent els punts aleatoris + GRTS
</commit_message>
<xml_diff>
--- a/Hores_feina.xlsx
+++ b/Hores_feina.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubarcelona-my.sharepoint.com/personal/vcarnele7_alumnes_ub_edu/Documents/Feina/UB/Carto/Seguiment_habitats/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuari\OneDrive - Universitat de Barcelona (2)\Feina\UB\Carto\Seguiment_habitats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="14_{AAB7CBA6-E2CE-4554-A50D-46C979D8C302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D14AEF58-CADD-5543-B8F6-71F8EACBF441}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="14_{9C64D7FB-523E-486C-AF3F-34B773B87610}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{3700CF86-494E-4F88-B43E-9E28C44D2689}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="500" windowWidth="28800" windowHeight="12160" xr2:uid="{ABC30D23-9473-424B-A90E-98722AE03216}"/>
+    <workbookView xWindow="0" yWindow="495" windowWidth="15360" windowHeight="6990" xr2:uid="{ABC30D23-9473-424B-A90E-98722AE03216}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,12 +23,6 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -102,9 +96,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -142,7 +136,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -248,7 +242,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -390,7 +384,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -398,10 +392,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E32FD3E7-A30A-4C80-B783-A22AB56124D0}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -412,7 +406,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46043</v>
       </c>
@@ -427,7 +421,7 @@
         <v>0.16666666666666669</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46043</v>
       </c>
@@ -438,11 +432,11 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="D3" s="2">
-        <f t="shared" ref="D3:D10" si="0">C3-B3</f>
+        <f t="shared" ref="D3:D15" si="0">C3-B3</f>
         <v>0.10416666666666674</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>46044</v>
       </c>
@@ -457,7 +451,7 @@
         <v>0.10416666666666669</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>46044</v>
       </c>
@@ -472,7 +466,7 @@
         <v>0.16666666666666663</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46045</v>
       </c>
@@ -487,7 +481,7 @@
         <v>8.3333333333333315E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>46045</v>
       </c>
@@ -502,7 +496,7 @@
         <v>0.10416666666666663</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>46048</v>
       </c>
@@ -517,7 +511,7 @@
         <v>0.16666666666666663</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>46049</v>
       </c>
@@ -532,7 +526,7 @@
         <v>8.333333333333337E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>46049</v>
       </c>
@@ -545,6 +539,81 @@
       <c r="D10" s="2">
         <f t="shared" si="0"/>
         <v>8.333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46052</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D11" s="2">
+        <f t="shared" si="0"/>
+        <v>8.3333333333333259E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>46055</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" si="0"/>
+        <v>8.333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46055</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D13" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>46056</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="D14" s="2">
+        <f t="shared" si="0"/>
+        <v>8.333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>46057</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="D15" s="2">
+        <f t="shared" si="0"/>
+        <v>6.25E-2</v>
       </c>
     </row>
   </sheetData>
@@ -553,6 +622,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E6C750F080D38148A6E2E1F0D59240B8" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a249966b2616fb475cd34c938a4c3752">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="a4f05a8b-6c99-4fde-9c58-e847a1350398" xmlns:ns4="c4bef083-dd18-488d-8b49-2edaf9c952e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3241f162b182046b53c2dc5bb106ce6b" ns3:_="" ns4:_="">
     <xsd:import namespace="a4f05a8b-6c99-4fde-9c58-e847a1350398"/>
@@ -799,15 +877,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -815,6 +884,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{219A7091-3CEF-46D1-9B3E-B230069E3FF5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3B738BF-43A1-4DE3-886B-F4B6154A7C5A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -833,27 +910,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{219A7091-3CEF-46D1-9B3E-B230069E3FF5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55060E34-C54B-467B-859E-BB6BC610DA27}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="c4bef083-dd18-488d-8b49-2edaf9c952e6"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="c4bef083-dd18-488d-8b49-2edaf9c952e6"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="a4f05a8b-6c99-4fde-9c58-e847a1350398"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>